<commit_message>
Show Shopify countries and hide daily averages in PYG workbooks
</commit_message>
<xml_diff>
--- a/output/spreadsheet/pyg_inc_2026.xlsx
+++ b/output/spreadsheet/pyg_inc_2026.xlsx
@@ -709,7 +709,7 @@
     <row r="3" ht="12" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Shopify daily average | Actualizado: 31/07/2026 09:48 h</t>
+          <t>Shopify daily average | Actualizado: 31/07/2026 12:25 h</t>
         </is>
       </c>
       <c r="B3" s="4" t="n"/>
@@ -955,7 +955,7 @@
         </is>
       </c>
     </row>
-    <row r="7" hidden="1" outlineLevel="3" ht="12" customHeight="1">
+    <row r="7" ht="12" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
           <t xml:space="preserve">      US</t>
@@ -1021,7 +1021,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="12" customHeight="1">
+    <row r="8" hidden="1" outlineLevel="3" ht="12" customHeight="1">
       <c r="A8" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">        avg/day</t>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-31T07:48:06Z</t>
+          <t>2026-07-31T10:25:42Z</t>
         </is>
       </c>
     </row>

</xml_diff>